<commit_message>
adjust user and aging add fimoco menu FBB
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -1,113 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BOT\pt3bot\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA8F2C8-B9B9-4424-9D5B-F3F335B3DB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="users" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="users" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
-  <si>
-    <t>nik</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>password_hash</t>
-  </si>
-  <si>
-    <t>role</t>
-  </si>
-  <si>
-    <t>project</t>
-  </si>
-  <si>
-    <t>10000001</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>scrypt:32768:8:1$YvC835gbNk6xd9sy$87f7fc4a0d8cb59f5c542e89ac603d838d252c68f2fd6326e5430d83d72f5b14adcc944f6c64a095376656b274a90e103817db17fdaa2980e7adc22b19b98fcd</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>ALL</t>
-  </si>
-  <si>
-    <t>10000002</t>
-  </si>
-  <si>
-    <t>Developer</t>
-  </si>
-  <si>
-    <t>scrypt:32768:8:1$Awop6owzwcxDsIry$805a02a3c6baf4e1c45ebe4c4d06f59aa33587657e95c48bb43bccf759596cae189f7631a78c0ec91d23916d0326a201baf66c041176ce49644cdabeb2e3e5db</t>
-  </si>
-  <si>
-    <t>developer</t>
-  </si>
-  <si>
-    <t>90000001</t>
-  </si>
-  <si>
-    <t>scrypt:32768:8:1$WkcVTPGf6uD3Q0Gn$17e9982d99fd4b48e8e984e1e63b746bc225d8bafeee9b692bcf140e57bd1bdab03f3348e0cfd1c0c74c4ec4f7335bc7c8adb91aa825a51b939131281cba3e4f</t>
-  </si>
-  <si>
-    <t>viewer</t>
-  </si>
-  <si>
-    <t>TIF &amp;Telkomsel</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -126,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -428,83 +408,154 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="95" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nik</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>password_hash</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>10000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Telkom Akses</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$3q2tuoD9uY7WP9eX$56e7552bcf75f054dc528bbbf4e446803f72539d62e08943a74066fe3f3157223dd49410757a1bc8291c7025571546591c9857c0f5ad771399844be4ce38ba12</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Edjabar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$ZEX8WKewqLBwgtDE$ac53b7a3be5f5f93be23cb1d914dc879bd9a4c813a9d247427c98730408db5364efacd63c475795ee5d3721e2ea523fbaab9a7a88ecf3b7017af41455ff9f461</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>90000001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Telkomsel</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$Xs36w8i4v0dvMQrv$90a46003624ac58c62872f3c47019fa687e192004ec8dacb77e2251a4a2e55803aef5c5f4b4b0c1ae7f840a2cca52963fb9296f94be563f33ea675857cf3b8ee</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10000003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$lgeF2Xl4WDVlZ9op$49867daf9f014ef5db9ef6f8335948bf6ac31a5f7f5a3c9ab44d20d08e605a346f573f42d7a5d04d082b3c84d7f90c4a6b485b2a2c1d275c3bc0fa0ec6947dca</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>developer</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>